<commit_message>
Indicate the parts that can be 3D printed no matter the materials purchased
</commit_message>
<xml_diff>
--- a/CAD/3d_print.xlsx
+++ b/CAD/3d_print.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\satom\Desktop\Robot\CAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA9C376F-5299-48B4-B498-BDDD7B4C3628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C7BCBD-EDD0-4E2B-BC14-1E6DC86F17DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="7530" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
   <si>
     <t>File Name</t>
   </si>
@@ -108,6 +108,12 @@
   </si>
   <si>
     <t>Filament (g, Total)</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>* = Can 3D print right now, does not depend on the materials purchased</t>
   </si>
 </sst>
 </file>
@@ -444,7 +450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="30.20703125" bestFit="1" customWidth="1"/>
@@ -454,7 +460,7 @@
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="3" t="s">
         <v>22</v>
       </c>
@@ -462,7 +468,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -479,7 +485,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -491,15 +497,15 @@
         <v>21.56</v>
       </c>
       <c r="D4">
-        <f>B4*$B$1</f>
+        <f t="shared" ref="D4:D20" si="0">B4*$B$1</f>
         <v>8</v>
       </c>
       <c r="E4">
-        <f>C4*$B$1</f>
+        <f t="shared" ref="E4:E20" si="1">C4*$B$1</f>
         <v>86.24</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -511,15 +517,15 @@
         <v>24.6</v>
       </c>
       <c r="D5">
-        <f>B5*$B$1</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="E5">
-        <f>C5*$B$1</f>
+        <f t="shared" si="1"/>
         <v>98.4</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -531,15 +537,15 @@
         <v>7.8</v>
       </c>
       <c r="D6">
-        <f>B6*$B$1</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="E6">
-        <f>C6*$B$1</f>
+        <f t="shared" si="1"/>
         <v>31.2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -551,15 +557,18 @@
         <v>35.200000000000003</v>
       </c>
       <c r="D7">
-        <f>B7*$B$1</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="E7">
-        <f>C7*$B$1</f>
+        <f t="shared" si="1"/>
         <v>140.80000000000001</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -571,15 +580,18 @@
         <v>24.02</v>
       </c>
       <c r="D8">
-        <f>B8*$B$1</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="E8">
-        <f>C8*$B$1</f>
+        <f t="shared" si="1"/>
         <v>96.08</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -591,15 +603,18 @@
         <v>24.78</v>
       </c>
       <c r="D9">
-        <f>B9*$B$1</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="E9">
-        <f>C9*$B$1</f>
+        <f t="shared" si="1"/>
         <v>99.12</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -611,15 +626,18 @@
         <v>6.5</v>
       </c>
       <c r="D10">
-        <f>B10*$B$1</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="E10">
-        <f>C10*$B$1</f>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -631,15 +649,18 @@
         <v>6.5</v>
       </c>
       <c r="D11">
-        <f>B11*$B$1</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="E11">
-        <f>C11*$B$1</f>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -651,15 +672,18 @@
         <v>351.36</v>
       </c>
       <c r="D12">
-        <f>B12*$B$1</f>
+        <f t="shared" si="0"/>
         <v>48</v>
       </c>
       <c r="E12">
-        <f>C12*$B$1</f>
+        <f t="shared" si="1"/>
         <v>1405.44</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -670,15 +694,15 @@
         <v>25.12</v>
       </c>
       <c r="D13">
-        <f>B13*$B$1</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="E13">
-        <f>C13*$B$1</f>
+        <f t="shared" si="1"/>
         <v>100.48</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -690,15 +714,18 @@
         <v>19.84</v>
       </c>
       <c r="D14">
-        <f>B14*$B$1</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="E14">
-        <f>C14*$B$1</f>
+        <f t="shared" si="1"/>
         <v>79.36</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -709,15 +736,15 @@
         <v>1.7</v>
       </c>
       <c r="D15">
-        <f>B15*$B$1</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="E15">
-        <f>C15*$B$1</f>
+        <f t="shared" si="1"/>
         <v>6.8</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
         <v>6</v>
       </c>
@@ -728,11 +755,11 @@
         <v>1.7</v>
       </c>
       <c r="D16">
-        <f>B16*$B$1</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="E16">
-        <f>C16*$B$1</f>
+        <f t="shared" si="1"/>
         <v>6.8</v>
       </c>
     </row>
@@ -747,11 +774,11 @@
         <v>6.27</v>
       </c>
       <c r="D17">
-        <f>B17*$B$1</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="E17">
-        <f>C17*$B$1</f>
+        <f t="shared" si="1"/>
         <v>25.08</v>
       </c>
     </row>
@@ -766,11 +793,11 @@
         <v>6.27</v>
       </c>
       <c r="D18">
-        <f>B18*$B$1</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="E18">
-        <f>C18*$B$1</f>
+        <f t="shared" si="1"/>
         <v>25.08</v>
       </c>
     </row>
@@ -786,11 +813,11 @@
         <v>5.42</v>
       </c>
       <c r="D19">
-        <f>B19*$B$1</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="E19">
-        <f>C19*$B$1</f>
+        <f t="shared" si="1"/>
         <v>21.68</v>
       </c>
     </row>
@@ -806,11 +833,11 @@
         <v>2.84</v>
       </c>
       <c r="D20">
-        <f>B20*$B$1</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="E20">
-        <f>C20*$B$1</f>
+        <f t="shared" si="1"/>
         <v>11.36</v>
       </c>
     </row>
@@ -827,6 +854,11 @@
       <c r="E21" s="2">
         <f>SUM(E4:E20)</f>
         <v>2285.92</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A23" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add details about bearing block with flanged vs non flanged bearings
</commit_message>
<xml_diff>
--- a/CAD/3d_print.xlsx
+++ b/CAD/3d_print.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\satom\Desktop\Robot\CAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C7BCBD-EDD0-4E2B-BC14-1E6DC86F17DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C503BA5-2257-4E3B-A4BF-D51F1761776C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="27">
   <si>
     <t>File Name</t>
   </si>
@@ -71,9 +71,6 @@
     <t>microphone_casing.STL</t>
   </si>
   <si>
-    <t>wheel_bearing_block.STL</t>
-  </si>
-  <si>
     <t>Quantity/Robot</t>
   </si>
   <si>
@@ -114,6 +111,12 @@
   </si>
   <si>
     <t>* = Can 3D print right now, does not depend on the materials purchased</t>
+  </si>
+  <si>
+    <t>wheel_bearing_block.STL OR wheel_bearing_block_no_flange.STL</t>
+  </si>
+  <si>
+    <t>&gt;&gt;&gt; Select the correct file depending on if your ball bearings have flanges or not</t>
   </si>
 </sst>
 </file>
@@ -453,7 +456,7 @@
   <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="30.20703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="57.578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25.05078125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.89453125" bestFit="1" customWidth="1"/>
@@ -462,7 +465,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B1">
         <v>4</v>
@@ -473,16 +476,16 @@
         <v>0</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="E3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -507,7 +510,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -524,6 +527,9 @@
         <f t="shared" si="1"/>
         <v>98.4</v>
       </c>
+      <c r="F5" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
@@ -565,12 +571,12 @@
         <v>140.80000000000001</v>
       </c>
       <c r="F7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8">
         <v>2</v>
@@ -588,12 +594,12 @@
         <v>96.08</v>
       </c>
       <c r="F8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9">
         <v>2</v>
@@ -611,12 +617,12 @@
         <v>99.12</v>
       </c>
       <c r="F9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B10">
         <v>2</v>
@@ -634,12 +640,12 @@
         <v>26</v>
       </c>
       <c r="F10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B11">
         <v>2</v>
@@ -657,12 +663,12 @@
         <v>26</v>
       </c>
       <c r="F11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B12">
         <v>12</v>
@@ -680,7 +686,7 @@
         <v>1405.44</v>
       </c>
       <c r="F12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -704,7 +710,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B14">
         <v>4</v>
@@ -722,7 +728,7 @@
         <v>79.36</v>
       </c>
       <c r="F14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -843,7 +849,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2">
@@ -858,7 +864,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add markdown for 3d printed parts
</commit_message>
<xml_diff>
--- a/CAD/3d_print.xlsx
+++ b/CAD/3d_print.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\satom\Desktop\Robot\CAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C503BA5-2257-4E3B-A4BF-D51F1761776C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC3EBA7F-2216-465F-A749-5E124A83D9BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11442" yWindow="0" windowWidth="11676" windowHeight="12318" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>